<commit_message>
Refine FOLU comment labels and method section
</commit_message>
<xml_diff>
--- a/data/folu_social_listening_report.xlsx
+++ b/data/folu_social_listening_report.xlsx
@@ -59954,7 +59954,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-16 02:22:15 +0700</t>
+          <t>2026-06-16 22:15:17 +0700</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -59989,7 +59989,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>{'instagram': 'BYOB + Instagram API/session scrape available from prior task; comments included.', 'youtube': 'YouTube streams/comments dataset included from prior scrape.', 'tiktok': 'BYOB discovery worked; Obscura attempted but returned blank/eval null on TikTok; fallback extractor/API/session used; comments included.', 'website': 'BYOB verified seeds + Obscura bulk text; zero-byte PPID pages excluded during cleaning.'}</t>
+          <t>{'instagram': 'Post dan komentar publik dinormalisasi dari halaman/reel relevan, termasuk metadata waktu, engagement, caption, dan URL.', 'youtube': 'Komentar dan metadata video disatukan ke skema lintas platform untuk analisis sentiment, topik, dan risk flag.', 'tiktok': 'Metadata post dan komentar diekstrak dari halaman publik, lalu dibersihkan dari duplikasi dan komentar low-information.', 'website': 'Artikel/halaman web relevan dipakai sebagai konteks media discourse; halaman kosong atau tidak valid dikeluarkan saat cleaning.'}</t>
         </is>
       </c>
     </row>

</xml_diff>